<commit_message>
Solved 1. Two Sum
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7532EB68-F0BB-4C1B-9640-F832374B87ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5914F0B7-C92F-4262-846E-DDAF20EBD51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8508" yWindow="1836" windowWidth="14340" windowHeight="8856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>Category</t>
   </si>
@@ -106,6 +106,15 @@
   </si>
   <si>
     <t>discrete binary search, 2D arrays;</t>
+  </si>
+  <si>
+    <t>Hash Table</t>
+  </si>
+  <si>
+    <t>Two Sum</t>
+  </si>
+  <si>
+    <t>hash table, value:ind;</t>
   </si>
 </sst>
 </file>
@@ -460,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -578,6 +587,17 @@
         <v>26</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 217. Contains Duplicate
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5914F0B7-C92F-4262-846E-DDAF20EBD51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B0B10C-5878-4FB6-A5A6-5EBC9838EDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8508" yWindow="1836" windowWidth="14340" windowHeight="8856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>Category</t>
   </si>
@@ -115,6 +115,12 @@
   </si>
   <si>
     <t>hash table, value:ind;</t>
+  </si>
+  <si>
+    <t>Contains Duplicate</t>
+  </si>
+  <si>
+    <t>hash table, set;</t>
   </si>
 </sst>
 </file>
@@ -469,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -598,6 +604,17 @@
         <v>29</v>
       </c>
     </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 242. Valid Anagram
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B0B10C-5878-4FB6-A5A6-5EBC9838EDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33BC21A-CFFD-486B-9901-07BF92CD445E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
   <si>
     <t>Category</t>
   </si>
@@ -120,7 +120,13 @@
     <t>Contains Duplicate</t>
   </si>
   <si>
-    <t>hash table, set;</t>
+    <t>Valid Anagram</t>
+  </si>
+  <si>
+    <t>hash table, unordered_map;</t>
+  </si>
+  <si>
+    <t>hash table, unordered_set;</t>
   </si>
 </sst>
 </file>
@@ -475,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -612,7 +618,18 @@
         <v>30</v>
       </c>
       <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated 1. Two Sum
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33BC21A-CFFD-486B-9901-07BF92CD445E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8BE387-6B43-4E38-B563-BECB737FC16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,19 +114,19 @@
     <t>Two Sum</t>
   </si>
   <si>
-    <t>hash table, value:ind;</t>
-  </si>
-  <si>
     <t>Contains Duplicate</t>
   </si>
   <si>
     <t>Valid Anagram</t>
   </si>
   <si>
-    <t>hash table, unordered_map;</t>
-  </si>
-  <si>
     <t>hash table, unordered_set;</t>
+  </si>
+  <si>
+    <t>hash table, unordered_map, value:ind;</t>
+  </si>
+  <si>
+    <t>hash table, unordered_map, char:cnt;</t>
   </si>
 </sst>
 </file>
@@ -607,7 +607,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -615,10 +615,10 @@
         <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -626,10 +626,10 @@
         <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved 49. Group Anagrams
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8BE387-6B43-4E38-B563-BECB737FC16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685ED200-A864-4CAB-8D13-80548897FC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>Category</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>hash table, unordered_map, char:cnt;</t>
+  </si>
+  <si>
+    <t>Group Anagrams</t>
+  </si>
+  <si>
+    <t>hash table, unordered_map, count array, array -&gt; string hash, string:{string, string, …};</t>
   </si>
 </sst>
 </file>
@@ -481,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -632,6 +638,17 @@
         <v>33</v>
       </c>
     </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 347. Top K Frequent Elements
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685ED200-A864-4CAB-8D13-80548897FC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4238E37B-C9B6-448D-BE4A-95978C545EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
   <si>
     <t>Category</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>hash table, unordered_map, count array, array -&gt; string hash, string:{string, string, …};</t>
+  </si>
+  <si>
+    <t>Top K Frequent Elements</t>
+  </si>
+  <si>
+    <t>hash table, map, bucket sort, freq:{int, int, …}; min_heap -&gt; cnt:num;</t>
   </si>
 </sst>
 </file>
@@ -487,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -649,6 +655,17 @@
         <v>35</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 238. Product of Array Except Self
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4238E37B-C9B6-448D-BE4A-95978C545EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E73E52-4708-4DAD-9C99-708FC795ACD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>Category</t>
   </si>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>hash table, map, bucket sort, freq:{int, int, …}; min_heap -&gt; cnt:num;</t>
+  </si>
+  <si>
+    <t>Product of Array Except Self</t>
+  </si>
+  <si>
+    <t>prefix, suffix, product; in-place, postfix;</t>
   </si>
 </sst>
 </file>
@@ -493,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -666,6 +672,17 @@
         <v>37</v>
       </c>
     </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated 125. Valid Palindrome
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEEB11FC-C6EB-4071-8306-35240D06ED17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA94E60C-E05F-418B-B6C6-567B1A467F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>Valid Palindrome</t>
   </si>
   <si>
-    <t>two pointers, string;</t>
-  </si>
-  <si>
     <t>Sorting</t>
   </si>
   <si>
@@ -151,6 +148,9 @@
   </si>
   <si>
     <t>hash table, unordered_set, index;</t>
+  </si>
+  <si>
+    <t>two pointers, string, isalnum(), tolower();</t>
   </si>
 </sst>
 </file>
@@ -554,128 +554,128 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" t="s">
         <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
         <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" t="s">
         <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
         <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
         <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
         <v>34</v>
-      </c>
-      <c r="C14" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
         <v>36</v>
-      </c>
-      <c r="C15" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -683,21 +683,21 @@
         <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" t="s">
         <v>38</v>
-      </c>
-      <c r="C16" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
         <v>40</v>
-      </c>
-      <c r="C17" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved 167. Two Sum II - Input Array is Sorted
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA94E60C-E05F-418B-B6C6-567B1A467F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2142E16C-5164-428A-9858-2B6D72650B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
   <si>
     <t>Category</t>
   </si>
@@ -151,6 +151,12 @@
   </si>
   <si>
     <t>two pointers, string, isalnum(), tolower();</t>
+  </si>
+  <si>
+    <t>Two Sum II - Input Array is Sorted</t>
+  </si>
+  <si>
+    <t>two pointers;</t>
   </si>
 </sst>
 </file>
@@ -505,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -700,6 +706,17 @@
         <v>40</v>
       </c>
     </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 128. Longest Consecutive Sequence
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2142E16C-5164-428A-9858-2B6D72650B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE8F7955-1F1D-49F6-9C72-88A7544BD78A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>Category</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t>two pointers;</t>
+  </si>
+  <si>
+    <t>Longest Consecutive Sequence</t>
+  </si>
+  <si>
+    <t>hash table, unordered_map, ranges; unordered_set, start;</t>
   </si>
 </sst>
 </file>
@@ -511,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -717,6 +723,17 @@
         <v>43</v>
       </c>
     </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 11. Container With Most Water
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE74BEFD-070B-489A-B8BA-0F526F14E811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F2F9FB-8DC0-49EB-B8E0-7AAA28D2024D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t>Category</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>two pointers, bruteforce, sort, no duplicates;</t>
+  </si>
+  <si>
+    <t>Container With Most Water</t>
+  </si>
+  <si>
+    <t>two pointers, min, greedy;</t>
   </si>
 </sst>
 </file>
@@ -523,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -751,6 +757,17 @@
         <v>47</v>
       </c>
     </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 1929. Concatenation of Array
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F2F9FB-8DC0-49EB-B8E0-7AAA28D2024D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E900B0-2033-4B4B-B2BA-D9F8C3436A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
   <si>
     <t>Category</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>two pointers, min, greedy;</t>
+  </si>
+  <si>
+    <t>Concatenation of Array</t>
+  </si>
+  <si>
+    <t>arrays;</t>
   </si>
 </sst>
 </file>
@@ -529,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -768,6 +774,17 @@
         <v>49</v>
       </c>
     </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 14. Longest Common Prefix
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E900B0-2033-4B4B-B2BA-D9F8C3436A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76671141-2071-481A-AF30-691A30EB033A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
   <si>
     <t>Category</t>
   </si>
@@ -181,6 +181,12 @@
   </si>
   <si>
     <t>arrays;</t>
+  </si>
+  <si>
+    <t>Longest Common Prefix</t>
+  </si>
+  <si>
+    <t>arrays, brute force, pass;</t>
   </si>
 </sst>
 </file>
@@ -535,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -785,6 +791,17 @@
         <v>51</v>
       </c>
     </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 122. Best Time to Buy and Sell Stock II
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76671141-2071-481A-AF30-691A30EB033A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E22CC9B-D452-4874-87A7-F17DBB65634E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
   <si>
     <t>Category</t>
   </si>
@@ -187,6 +187,12 @@
   </si>
   <si>
     <t>arrays, brute force, pass;</t>
+  </si>
+  <si>
+    <t>Best Time to Buy and Sell Stock II</t>
+  </si>
+  <si>
+    <t>arrays, greedy;</t>
   </si>
 </sst>
 </file>
@@ -541,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -802,6 +808,17 @@
         <v>53</v>
       </c>
     </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 560. Subarray Sum Equals K
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E22CC9B-D452-4874-87A7-F17DBB65634E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30276AC-3CBB-4F32-8149-3BCB801AD785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
   <si>
     <t>Category</t>
   </si>
@@ -193,6 +193,12 @@
   </si>
   <si>
     <t>arrays, greedy;</t>
+  </si>
+  <si>
+    <t>Subarray Sum Equals K</t>
+  </si>
+  <si>
+    <t>prefix, hash table, freq;</t>
   </si>
 </sst>
 </file>
@@ -547,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -819,6 +825,17 @@
         <v>55</v>
       </c>
     </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 680. Valid Palindrome II
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30276AC-3CBB-4F32-8149-3BCB801AD785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16560E37-844C-421A-8F58-D5C9E8EFA0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
   <si>
     <t>Category</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>prefix, hash table, freq;</t>
+  </si>
+  <si>
+    <t>Valid Palindrome II</t>
+  </si>
+  <si>
+    <t>two pointers, greedy;</t>
   </si>
 </sst>
 </file>
@@ -553,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -836,6 +842,17 @@
         <v>57</v>
       </c>
     </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 881. Boats to Save People
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16560E37-844C-421A-8F58-D5C9E8EFA0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B009D23-9AF3-443C-A142-40D84557CC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="62">
   <si>
     <t>Category</t>
   </si>
@@ -205,6 +205,12 @@
   </si>
   <si>
     <t>two pointers, greedy;</t>
+  </si>
+  <si>
+    <t>Boats to Save People</t>
+  </si>
+  <si>
+    <t>two pointers, sort, greedy; counting sort;</t>
   </si>
 </sst>
 </file>
@@ -559,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -853,6 +859,17 @@
         <v>59</v>
       </c>
     </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 42. Trapping Rain Water
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B009D23-9AF3-443C-A142-40D84557CC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67091452-29B3-45A9-8E53-171512F70896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
   <si>
     <t>Category</t>
   </si>
@@ -211,13 +211,19 @@
   </si>
   <si>
     <t>two pointers, sort, greedy; counting sort;</t>
+  </si>
+  <si>
+    <t>Trapping Rain Water</t>
+  </si>
+  <si>
+    <t>two pointers, ind, max; prefix, suffix, max;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,8 +253,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF800000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,6 +280,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF5050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -280,17 +299,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF5050"/>
+      <color rgb="FF800000"/>
+      <color rgb="FFD00000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -565,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -870,6 +897,17 @@
         <v>61</v>
       </c>
     </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 121. Best Time to Buy and Sell Stock
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67091452-29B3-45A9-8E53-171512F70896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E195986E-59BF-448A-A9C8-967B9455A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
   <si>
     <t>Category</t>
   </si>
@@ -217,6 +217,15 @@
   </si>
   <si>
     <t>two pointers, ind, max; prefix, suffix, max;</t>
+  </si>
+  <si>
+    <t>Sliding Window</t>
+  </si>
+  <si>
+    <t>Best Time to Buy and Sell Stock</t>
+  </si>
+  <si>
+    <t>sliding window; dp;</t>
   </si>
 </sst>
 </file>
@@ -592,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -908,6 +917,17 @@
         <v>63</v>
       </c>
     </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 3. Longest Substring Without Repeating Characters
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E195986E-59BF-448A-A9C8-967B9455A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF97DEA8-5E5A-481E-BA9C-BFBCCF2C79A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
   <si>
     <t>Category</t>
   </si>
@@ -226,6 +226,12 @@
   </si>
   <si>
     <t>sliding window; dp;</t>
+  </si>
+  <si>
+    <t>Longest Substring Without Repeating Characters</t>
+  </si>
+  <si>
+    <t>sliding window, hash table, ind;</t>
   </si>
 </sst>
 </file>
@@ -601,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -928,6 +934,17 @@
         <v>66</v>
       </c>
     </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 20. Valid Parentheses
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF97DEA8-5E5A-481E-BA9C-BFBCCF2C79A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C39784-D96E-4FD5-9C53-438872EA4F52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="72">
   <si>
     <t>Category</t>
   </si>
@@ -232,6 +232,15 @@
   </si>
   <si>
     <t>sliding window, hash table, ind;</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Valid Parentheses</t>
+  </si>
+  <si>
+    <t>stack, hash table;</t>
   </si>
 </sst>
 </file>
@@ -607,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -945,6 +954,17 @@
         <v>68</v>
       </c>
     </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 150. Evaluate Reverse Polish Notation
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15C39784-D96E-4FD5-9C53-438872EA4F52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7AA95CB-5B19-4867-9F49-ED5F4ED8AC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
   <si>
     <t>Category</t>
   </si>
@@ -241,6 +241,12 @@
   </si>
   <si>
     <t>stack, hash table;</t>
+  </si>
+  <si>
+    <t>Evaluate Reverse Polish Notation</t>
+  </si>
+  <si>
+    <t>stack, stoi;</t>
   </si>
 </sst>
 </file>
@@ -616,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -965,6 +971,17 @@
         <v>71</v>
       </c>
     </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 70. Climbing Stairs
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7AA95CB-5B19-4867-9F49-ED5F4ED8AC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D826D3ED-9836-4638-9C41-76E8BEFEF55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
   <si>
     <t>Category</t>
   </si>
@@ -247,6 +247,15 @@
   </si>
   <si>
     <t>stack, stoi;</t>
+  </si>
+  <si>
+    <t>DP 1-D</t>
+  </si>
+  <si>
+    <t>Climbing Stairs</t>
+  </si>
+  <si>
+    <t>dp 1-D;</t>
   </si>
 </sst>
 </file>
@@ -622,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -982,6 +991,17 @@
         <v>73</v>
       </c>
     </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 198. House Robber
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D826D3ED-9836-4638-9C41-76E8BEFEF55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E4491C-03A0-4A9D-8C90-145431E1DA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="2004" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="79">
   <si>
     <t>Category</t>
   </si>
@@ -256,6 +256,12 @@
   </si>
   <si>
     <t>dp 1-D;</t>
+  </si>
+  <si>
+    <t>House Robber</t>
+  </si>
+  <si>
+    <t>dp 1-D; dfs, memoization;</t>
   </si>
 </sst>
 </file>
@@ -631,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1002,6 +1008,17 @@
         <v>76</v>
       </c>
     </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" t="s">
+        <v>78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 424. Longest Repeating Character Replacement
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E4491C-03A0-4A9D-8C90-145431E1DA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091CC650-66BD-4559-A59B-E9748E603DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3708" yWindow="2352" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="81">
   <si>
     <t>Category</t>
   </si>
@@ -262,6 +262,12 @@
   </si>
   <si>
     <t>dp 1-D; dfs, memoization;</t>
+  </si>
+  <si>
+    <t>Longest Repeating Character Replacement</t>
+  </si>
+  <si>
+    <t>sliding window, hash table, cnt, max;</t>
   </si>
 </sst>
 </file>
@@ -637,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1019,6 +1025,17 @@
         <v>78</v>
       </c>
     </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 76. Minimum Window Substring
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091CC650-66BD-4559-A59B-E9748E603DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78412DB-471A-4CEE-AF2A-3DD376E30CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3708" yWindow="2352" windowWidth="19236" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="83">
   <si>
     <t>Category</t>
   </si>
@@ -268,6 +268,12 @@
   </si>
   <si>
     <t>sliding window, hash table, cnt, max;</t>
+  </si>
+  <si>
+    <t>Minimum Window Substring</t>
+  </si>
+  <si>
+    <t>sliding window, hash table, cnt, min;</t>
   </si>
 </sst>
 </file>
@@ -643,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1036,6 +1042,17 @@
         <v>80</v>
       </c>
     </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C36" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 153. Find Minimum in Rotated Sorted Array
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78412DB-471A-4CEE-AF2A-3DD376E30CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54534AF-9577-4C7B-8D5E-AB29A5E84766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="85">
   <si>
     <t>Category</t>
   </si>
@@ -274,6 +274,12 @@
   </si>
   <si>
     <t>sliding window, hash table, cnt, min;</t>
+  </si>
+  <si>
+    <t>Find Minimum in Rotated Sorted Array</t>
+  </si>
+  <si>
+    <t>discrete binary search, segments;</t>
   </si>
 </sst>
 </file>
@@ -649,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1053,6 +1059,17 @@
         <v>82</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 33. Search in Rotated Sorted Array
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54534AF-9577-4C7B-8D5E-AB29A5E84766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD80DD3-2EB8-4F7D-9055-71751458902B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
   <si>
     <t>Category</t>
   </si>
@@ -280,6 +280,12 @@
   </si>
   <si>
     <t>discrete binary search, segments;</t>
+  </si>
+  <si>
+    <t>discrete binary search, segments, two pass;</t>
+  </si>
+  <si>
+    <t>Search in Rotated Sorted Array</t>
   </si>
 </sst>
 </file>
@@ -655,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1070,6 +1076,17 @@
         <v>84</v>
       </c>
     </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 206. Reverse Linked List
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD80DD3-2EB8-4F7D-9055-71751458902B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632524B2-27DF-4D44-867A-5421AA4399FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
   <si>
     <t>Category</t>
   </si>
@@ -286,6 +286,15 @@
   </si>
   <si>
     <t>Search in Rotated Sorted Array</t>
+  </si>
+  <si>
+    <t>Linked List</t>
+  </si>
+  <si>
+    <t>Reverse Linked List</t>
+  </si>
+  <si>
+    <t>linked list iteration; recursive;</t>
   </si>
 </sst>
 </file>
@@ -661,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1087,6 +1096,17 @@
         <v>85</v>
       </c>
     </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 21. Merge Two Sorted Lists
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632524B2-27DF-4D44-867A-5421AA4399FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DDFE1B-EEFD-4EF9-97B8-B05E7DB52943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="92">
   <si>
     <t>Category</t>
   </si>
@@ -294,7 +294,13 @@
     <t>Reverse Linked List</t>
   </si>
   <si>
-    <t>linked list iteration; recursive;</t>
+    <t>linked list iteration; recursion;</t>
+  </si>
+  <si>
+    <t>linked list iteration, dummy; recursion;</t>
+  </si>
+  <si>
+    <t>Merge Two Sorted Lists</t>
   </si>
 </sst>
 </file>
@@ -670,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1107,6 +1113,17 @@
         <v>89</v>
       </c>
     </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 141. Linked List Cycle
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DDFE1B-EEFD-4EF9-97B8-B05E7DB52943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1AE970-DF3B-4CA8-83B0-ACD83798FB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="94">
   <si>
     <t>Category</t>
   </si>
@@ -301,6 +301,12 @@
   </si>
   <si>
     <t>Merge Two Sorted Lists</t>
+  </si>
+  <si>
+    <t>linked list iteration, unordered_set; fast &amp; slow pointers;</t>
+  </si>
+  <si>
+    <t>Linked List Cycle</t>
   </si>
 </sst>
 </file>
@@ -676,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1124,6 +1130,17 @@
         <v>90</v>
       </c>
     </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" t="s">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 143. Reorder List
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1AE970-DF3B-4CA8-83B0-ACD83798FB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831F1009-54CF-4A08-8B0E-ABE29C74ED7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="96">
   <si>
     <t>Category</t>
   </si>
@@ -307,6 +307,12 @@
   </si>
   <si>
     <t>Linked List Cycle</t>
+  </si>
+  <si>
+    <t>Reorder List</t>
+  </si>
+  <si>
+    <t>linked list reverse, fast &amp; slow pointers; recursion;</t>
   </si>
 </sst>
 </file>
@@ -682,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1141,6 +1147,17 @@
         <v>92</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C42" t="s">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 19. Remove Nth Node From End of List
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831F1009-54CF-4A08-8B0E-ABE29C74ED7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8C767E-A2B0-420E-A6EB-61CCC6D83767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="98">
   <si>
     <t>Category</t>
   </si>
@@ -313,6 +313,12 @@
   </si>
   <si>
     <t>linked list reverse, fast &amp; slow pointers; recursion;</t>
+  </si>
+  <si>
+    <t>Remove Nth Node From End of List</t>
+  </si>
+  <si>
+    <t>linked list iteration, two pass; greedy, two pointers;</t>
   </si>
 </sst>
 </file>
@@ -688,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1158,6 +1164,17 @@
         <v>95</v>
       </c>
     </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C43" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 23. Merge k Sorted Lists
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8C767E-A2B0-420E-A6EB-61CCC6D83767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0562944A-997E-460C-B5F2-B6CBBA3C6F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
   <si>
     <t>Category</t>
   </si>
@@ -319,6 +319,12 @@
   </si>
   <si>
     <t>linked list iteration, two pass; greedy, two pointers;</t>
+  </si>
+  <si>
+    <t>Merge k Sorted Lists</t>
+  </si>
+  <si>
+    <t>heap, cmp, mergesort;</t>
   </si>
 </sst>
 </file>
@@ -694,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1175,6 +1181,17 @@
         <v>97</v>
       </c>
     </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C44" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 226. Invert Binary Tree
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0562944A-997E-460C-B5F2-B6CBBA3C6F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2052A3D9-9D61-4CA4-8232-1FDDB27B887A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="103">
   <si>
     <t>Category</t>
   </si>
@@ -325,6 +325,15 @@
   </si>
   <si>
     <t>heap, cmp, mergesort;</t>
+  </si>
+  <si>
+    <t>Trees</t>
+  </si>
+  <si>
+    <t>Invert Binary Tree</t>
+  </si>
+  <si>
+    <t>trees, dfs;</t>
   </si>
 </sst>
 </file>
@@ -700,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1192,6 +1201,17 @@
         <v>99</v>
       </c>
     </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>100</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C45" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
104. Maximum Depth of Binary Tree
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2052A3D9-9D61-4CA4-8232-1FDDB27B887A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47179CE6-EFBC-42B9-8317-EEBDC391399E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="105">
   <si>
     <t>Category</t>
   </si>
@@ -333,7 +333,13 @@
     <t>Invert Binary Tree</t>
   </si>
   <si>
-    <t>trees, dfs;</t>
+    <t>Maximum Depth of Binary Tree</t>
+  </si>
+  <si>
+    <t>trees, dfs, max;</t>
+  </si>
+  <si>
+    <t>trees, dfs, swap;</t>
   </si>
 </sst>
 </file>
@@ -709,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1209,7 +1215,18 @@
         <v>101</v>
       </c>
       <c r="C45" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>100</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>102</v>
+      </c>
+      <c r="C46" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved 100. Same Tree
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47179CE6-EFBC-42B9-8317-EEBDC391399E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48794F9-A55F-493F-A189-D251AA9AE8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="107">
   <si>
     <t>Category</t>
   </si>
@@ -340,6 +340,12 @@
   </si>
   <si>
     <t>trees, dfs, swap;</t>
+  </si>
+  <si>
+    <t>Same Tree</t>
+  </si>
+  <si>
+    <t>trees, dfs, bool, nullptr;</t>
   </si>
 </sst>
 </file>
@@ -715,7 +721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1229,6 +1235,17 @@
         <v>103</v>
       </c>
     </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>100</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Solved 572. Subtree of Another Tree
</commit_message>
<xml_diff>
--- a/cheat sheet.xlsx
+++ b/cheat sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\alg\LeetCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48794F9-A55F-493F-A189-D251AA9AE8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79DA48F-196D-4B0B-B012-C1B0D1B4D47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="109">
   <si>
     <t>Category</t>
   </si>
@@ -346,6 +346,12 @@
   </si>
   <si>
     <t>trees, dfs, bool, nullptr;</t>
+  </si>
+  <si>
+    <t>Subtree of Another Tree</t>
+  </si>
+  <si>
+    <t>trees, dfs^2, bool, nullptr;</t>
   </si>
 </sst>
 </file>
@@ -721,7 +727,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" customWidth="1"/>
@@ -1246,6 +1252,17 @@
         <v>106</v>
       </c>
     </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C48" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>